<commit_message>
Complete Admin Portal with employee management, reports, progress, approvals and settings
</commit_message>
<xml_diff>
--- a/backend/InternTrack_Report.xlsx
+++ b/backend/InternTrack_Report.xlsx
@@ -397,351 +397,175 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:M4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>employeeId</v>
+      </c>
+      <c r="C1" t="str">
         <v>employeeName</v>
       </c>
-      <c r="B1" t="str">
+      <c r="D1" t="str">
+        <v>employeeEmail</v>
+      </c>
+      <c r="E1" t="str">
+        <v>department</v>
+      </c>
+      <c r="F1" t="str">
         <v>reportDate</v>
       </c>
-      <c r="C1" t="str">
+      <c r="G1" t="str">
         <v>task</v>
       </c>
-      <c r="D1" t="str">
+      <c r="H1" t="str">
+        <v>description</v>
+      </c>
+      <c r="I1" t="str">
         <v>progress</v>
       </c>
-      <c r="E1" t="str">
+      <c r="J1" t="str">
+        <v>hoursWorked</v>
+      </c>
+      <c r="K1" t="str">
         <v>status</v>
       </c>
-      <c r="F1" t="str">
-        <v>id</v>
+      <c r="L1" t="str">
+        <v>managerRemarks</v>
+      </c>
+      <c r="M1" t="str">
+        <v>submittedAt</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="str">
         <v>Hrithik</v>
       </c>
-      <c r="B2" t="str">
-        <v>2026-07-17</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Backend Testing</v>
-      </c>
       <c r="D2" t="str">
-        <v>Testing POST</v>
+        <v>hrithik@gmail.com</v>
       </c>
       <c r="E2" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F2">
-        <v>2</v>
+        <v>AI &amp; DS</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Employee Records Module</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Completed redesign of Employee Records page.</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Finished cards, search, archive and responsive layout.</v>
+      </c>
+      <c r="J2">
+        <v>8</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Excellent work.</v>
+      </c>
+      <c r="M2" t="str">
+        <v>2026-07-29T17:15:00</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>Ashwin</v>
-      </c>
-      <c r="B3" t="str">
-        <v>2026-07-14</v>
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
       </c>
       <c r="C3" t="str">
-        <v>web server testing</v>
+        <v>Bhuvana</v>
       </c>
       <c r="D3" t="str">
-        <v>checking if the local server works properly</v>
+        <v>bhuvana@gmail.com</v>
       </c>
       <c r="E3" t="str">
+        <v>Backend</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Reports API</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Worked on import and export APIs.</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Import API completed. Export testing pending.</v>
+      </c>
+      <c r="J3">
+        <v>7</v>
+      </c>
+      <c r="K3" t="str">
         <v>Pending</v>
       </c>
-      <c r="F3">
-        <v>3</v>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v>2026-07-29T18:00:00</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>Newton</v>
-      </c>
-      <c r="B4" t="str">
-        <v>2026-07-17</v>
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
       </c>
       <c r="C4" t="str">
-        <v>presentation</v>
+        <v>Aditya</v>
       </c>
       <c r="D4" t="str">
-        <v>completed the 2nd part of presentation</v>
+        <v>aditya@gmail.com</v>
       </c>
       <c r="E4" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Rahul</v>
-      </c>
-      <c r="B5" t="str">
-        <v>2026-07-17</v>
-      </c>
-      <c r="C5" t="str">
-        <v>documentaion</v>
-      </c>
-      <c r="D5" t="str">
-        <v>complete the excel documentation</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F5">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Aditya</v>
-      </c>
-      <c r="B6" t="str">
-        <v>2026-07-14</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Frontend</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Designed dashboard UI</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Pending</v>
-      </c>
-      <c r="F6">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Akshay</v>
-      </c>
-      <c r="B7" t="str">
-        <v>2026-07-18</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Email Validation</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Validated company emails</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F7">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Newton</v>
-      </c>
-      <c r="B8" t="str">
-        <v>2026-07-19</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Presentation</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Completed project presentation</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F8">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Hiba</v>
-      </c>
-      <c r="B9" t="str">
-        <v>2026-07-19</v>
-      </c>
-      <c r="C9" t="str">
-        <v>API Testing</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Verified all REST APIs</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F9">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Priya</v>
-      </c>
-      <c r="B10" t="str">
-        <v>2026-07-20</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Documentation</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Prepared API documentation</v>
-      </c>
-      <c r="E10" t="str">
-        <v>In Progress</v>
-      </c>
-      <c r="F10">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Aditya</v>
-      </c>
-      <c r="B11" t="str">
-        <v>2026-07-15</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Frontend</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Designed dashboard UI</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F11">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Karthi</v>
-      </c>
-      <c r="B12" t="str">
-        <v>2026-07-15</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Frontend</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Designed dashboard UI</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F12">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Ashik</v>
-      </c>
-      <c r="B13" t="str">
-        <v>2026-07-17</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Backend Testing</v>
-      </c>
-      <c r="D13" t="str">
-        <v>Tested POST API</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F13">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Kadhir</v>
-      </c>
-      <c r="B14" t="str">
-        <v>2026-07-18</v>
-      </c>
-      <c r="C14" t="str">
-        <v>API Integration</v>
-      </c>
-      <c r="D14" t="str">
-        <v>Connected frontend with backend</v>
-      </c>
-      <c r="E14" t="str">
-        <v>In Progress</v>
-      </c>
-      <c r="F14">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Kumar</v>
-      </c>
-      <c r="B15" t="str">
-        <v>2026-07-15</v>
-      </c>
-      <c r="C15" t="str">
-        <v>Frontend</v>
-      </c>
-      <c r="D15" t="str">
-        <v>Designed dashboard UI</v>
-      </c>
-      <c r="E15" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F15">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Neeraj</v>
-      </c>
-      <c r="B16" t="str">
-        <v>2026-07-22</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Emails</v>
-      </c>
-      <c r="D16" t="str">
-        <v>Verify emails and send valid responses</v>
-      </c>
-      <c r="E16" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F16">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>Vaishak</v>
-      </c>
-      <c r="B17" t="str">
-        <v>2026-07-23</v>
-      </c>
-      <c r="C17" t="str">
-        <v>Presentation</v>
-      </c>
-      <c r="D17" t="str">
-        <v>Presented regarding the new changes in layout</v>
-      </c>
-      <c r="E17" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="F17">
-        <v>31</v>
+        <v>UI/UX</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Dashboard UI</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Designed dashboard cards.</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Awaiting review.</v>
+      </c>
+      <c r="J4">
+        <v>6</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Rejected</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Please improve alignment.</v>
+      </c>
+      <c r="M4" t="str">
+        <v>2026-07-29T16:45:00</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>